<commit_message>
Red de actores: 40 nodos (10 complementarios por verificar) y 56 aristas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/red-actores-kennedy.xlsx
+++ b/datos/red-actores-kennedy.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="781">
   <si>
     <t>Codigo</t>
   </si>
@@ -1196,6 +1196,222 @@
     <t>-74.16252</t>
   </si>
   <si>
+    <t>ACT-INST-06</t>
+  </si>
+  <si>
+    <t>IDIGER (Instituto Distrital de Gestión de Riesgos y Cambio Climático)</t>
+  </si>
+  <si>
+    <t>UPZ 79 Calandaima · Drenaje y riesgo de inundación</t>
+  </si>
+  <si>
+    <t>Gestión del riesgo por inundación y encharcamiento en la cuenca del Tintal</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Media · Poder de decisión: Regulatorio / Emergencias</t>
+  </si>
+  <si>
+    <t>Coordinación: Interinstitucional · Acción: Respuesta y conceptos técnicos</t>
+  </si>
+  <si>
+    <t>Control de información: Mapas de amenaza</t>
+  </si>
+  <si>
+    <t>Complemento propuesto — por verificar en campo (coordenada aproximada)</t>
+  </si>
+  <si>
+    <t>ACT-INST-07</t>
+  </si>
+  <si>
+    <t>UAESP (Unidad Administrativa Especial de Servicios Públicos)</t>
+  </si>
+  <si>
+    <t>UPZ 80 Corabastos · Gestión de residuos y reciclaje</t>
+  </si>
+  <si>
+    <t>Política de aseo, aprovechamiento y reconocimiento de recicladores de oficio</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Baja · Poder de decisión: Regulatorio / Contractual</t>
+  </si>
+  <si>
+    <t>Coordinación: Interinstitucional · Acción: Contratos de aseo y ECAs</t>
+  </si>
+  <si>
+    <t>Control de información: Censo de recicladores</t>
+  </si>
+  <si>
+    <t>ACT-INST-08</t>
+  </si>
+  <si>
+    <t>IDU (Instituto de Desarrollo Urbano)</t>
+  </si>
+  <si>
+    <t>UPZ 80 Corabastos / UPZ 79 Calandaima · Obra vial</t>
+  </si>
+  <si>
+    <t>Construcción y mantenimiento de la malla vial arterial (Av. Ciudad de Cali, Av. Tintal)</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Baja · Poder de decisión: Operativo / Contractual</t>
+  </si>
+  <si>
+    <t>Coordinación: Con consorcios · Acción: Obra pública</t>
+  </si>
+  <si>
+    <t>Control de información: Diseños y presupuestos</t>
+  </si>
+  <si>
+    <t>ACT-CORP-04</t>
+  </si>
+  <si>
+    <t>Plataformas logísticas y bodegas del eje Tintal</t>
+  </si>
+  <si>
+    <t>UPZ 78 Tintal Norte · Zona de bodegaje</t>
+  </si>
+  <si>
+    <t>Almacenamiento y despacho de carga ligada a Corabastos y al eje industrial</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Muy Baja · Poder de decisión: Económico / Locativo</t>
+  </si>
+  <si>
+    <t>Coordinación: Gremial · Acción: Ocupación del suelo y tráfico pesado</t>
+  </si>
+  <si>
+    <t>Control de información: Privada</t>
+  </si>
+  <si>
+    <t>ACT-COM-08</t>
+  </si>
+  <si>
+    <t>Observadores de aves (Asociación Bogotana de Ornitología)</t>
+  </si>
+  <si>
+    <t>UPZ 79 Calandaima · Humedales de Kennedy</t>
+  </si>
+  <si>
+    <t>Monitoreo ciudadano de avifauna y ciencia participativa en los humedales</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Alta · Poder de decisión: Incidencia técnica</t>
+  </si>
+  <si>
+    <t>Coordinación: Red de observadores · Acción: Conteos y reportes</t>
+  </si>
+  <si>
+    <t>Control de información: Registros de avistamientos</t>
+  </si>
+  <si>
+    <t>ACT-COM-09</t>
+  </si>
+  <si>
+    <t>Biblioteca El Tintal (Manuel Zapata Olivella)</t>
+  </si>
+  <si>
+    <t>UPZ 79 Calandaima / Tintal · Equipamiento cultural</t>
+  </si>
+  <si>
+    <t>Equipamiento cultural y educativo vecino que acoge actividades de humedal</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Media · Poder de decisión: Programático</t>
+  </si>
+  <si>
+    <t>Coordinación: Con colectivos y colegios · Acción: Talleres y ferias</t>
+  </si>
+  <si>
+    <t>Control de información: Archivo público</t>
+  </si>
+  <si>
+    <t>ACT-BIO-10</t>
+  </si>
+  <si>
+    <t>Arbolado exótico de ronda (Eucalipto, Acacia, Pino)</t>
+  </si>
+  <si>
+    <t>UPZ 80 Corabastos · Rondas y separadores viales</t>
+  </si>
+  <si>
+    <t>Vegetación introducida que compite con la flora nativa y modifica el microclima</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Baja · Poder de decisión: Competencia por luz y agua</t>
+  </si>
+  <si>
+    <t>Coordinación: Ninguna · Acción: Sombra, hojarasca y consumo hídrico</t>
+  </si>
+  <si>
+    <t>Control de información: Inventario del arbolado</t>
+  </si>
+  <si>
+    <t>ACT-FIS-07</t>
+  </si>
+  <si>
+    <t>Canal Castilla y canales de drenaje pluvial</t>
+  </si>
+  <si>
+    <t>Tecnológica / Natural</t>
+  </si>
+  <si>
+    <t>UPZ 79 Calandaima / Castilla · Drenaje</t>
+  </si>
+  <si>
+    <t>Conduce las aguas lluvias hacia y desde los humedales y el río Bogotá</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Alta · Poder de decisión: Ninguno (infraestructura)</t>
+  </si>
+  <si>
+    <t>Coordinación: Con la red de la EAAB · Acción: Transporte de agua y sedimentos</t>
+  </si>
+  <si>
+    <t>Control de información: Redes de monitoreo EAAB</t>
+  </si>
+  <si>
+    <t>ACT-FIS-08</t>
+  </si>
+  <si>
+    <t>Reserva Humedal de Techo</t>
+  </si>
+  <si>
+    <t>UPZ 77 Zona Industrial / Techo · Humedal</t>
+  </si>
+  <si>
+    <t>Humedal vecino al norte, refugio y corredor para la avifauna de Kennedy</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Alta · Poder de decisión: Área protegida</t>
+  </si>
+  <si>
+    <t>Coordinación: Colectivos locales · Acción: Amortiguación hídrica y hábitat</t>
+  </si>
+  <si>
+    <t>Control de información: Estudios de la SDA</t>
+  </si>
+  <si>
+    <t>ACT-FIS-09</t>
+  </si>
+  <si>
+    <t>Corredor vial Av. Agoberto Mejía / Av. Tintal</t>
+  </si>
+  <si>
+    <t>UPZ 78 Tintal Norte / UPZ 82 · Eje vial</t>
+  </si>
+  <si>
+    <t>Eje de crecimiento urbano que valoriza el suelo de borde de humedal</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad territorial: Baja · Poder de decisión: Ninguno (infraestructura)</t>
+  </si>
+  <si>
+    <t>Coordinación: Con el IDU · Acción: Conecta y fragmenta</t>
+  </si>
+  <si>
+    <t>Control de información: Pública</t>
+  </si>
+  <si>
     <t>Origen</t>
   </si>
   <si>
@@ -1812,6 +2028,270 @@
   </si>
   <si>
     <t>Planes de reasentamiento Metro Bogotá</t>
+  </si>
+  <si>
+    <t>EDG-39</t>
+  </si>
+  <si>
+    <t>Normativa / Gestión del riesgo (Unidireccional)</t>
+  </si>
+  <si>
+    <t>IDIGER define las zonas de encharcamiento que dependen de la red de colectores y emite conceptos para obras de drenaje.</t>
+  </si>
+  <si>
+    <t>Alta: decide prioridades sin operar la red.</t>
+  </si>
+  <si>
+    <t>Mapas de amenaza por inundación</t>
+  </si>
+  <si>
+    <t>EDG-40</t>
+  </si>
+  <si>
+    <t>Regulatoria / Amortiguación (Unidireccional)</t>
+  </si>
+  <si>
+    <t>El humedal se reconoce como amortiguador de crecientes dentro de la gestión del riesgo de la cuenca.</t>
+  </si>
+  <si>
+    <t>Media: el reconocimiento no financia la conservación.</t>
+  </si>
+  <si>
+    <t>Conceptos técnicos del IDIGER</t>
+  </si>
+  <si>
+    <t>EDG-41</t>
+  </si>
+  <si>
+    <t>Normativa / Reconocimiento (Bidireccional)</t>
+  </si>
+  <si>
+    <t>La UAESP reconoce y registra a los recicladores de oficio, pero la remuneración depende de tarifas de aseo.</t>
+  </si>
+  <si>
+    <t>Alta: el registro condiciona el acceso a ingresos.</t>
+  </si>
+  <si>
+    <t>Censo de recicladores</t>
+  </si>
+  <si>
+    <t>EDG-42</t>
+  </si>
+  <si>
+    <t>Regulatoria / Residuos (Unidireccional)</t>
+  </si>
+  <si>
+    <t>La entidad define reglas de aprovechamiento de los residuos orgánicos y de cartón que genera la central.</t>
+  </si>
+  <si>
+    <t>Alta: la central externaliza parte de la gestión.</t>
+  </si>
+  <si>
+    <t>Plan de gestión de residuos</t>
+  </si>
+  <si>
+    <t>EDG-43</t>
+  </si>
+  <si>
+    <t>Administrativa / Obra vial (Unidireccional)</t>
+  </si>
+  <si>
+    <t>El IDU decide ensanches y mantenimiento que consolidan la calzada que parte el humedal.</t>
+  </si>
+  <si>
+    <t>Alta: la obra prima sobre la conectividad ecológica.</t>
+  </si>
+  <si>
+    <t>Contratos de obra vial</t>
+  </si>
+  <si>
+    <t>EDG-44</t>
+  </si>
+  <si>
+    <t>Logística / Carga (Bidireccional)</t>
+  </si>
+  <si>
+    <t>Las bodegas generan tráfico pesado sobre el corredor y presionan por más capacidad vial.</t>
+  </si>
+  <si>
+    <t>Alta: externalizan el costo del desgaste.</t>
+  </si>
+  <si>
+    <t>Aforos de carga pesada</t>
+  </si>
+  <si>
+    <t>EDG-45</t>
+  </si>
+  <si>
+    <t>Constructiva / Sellamiento (Unidireccional)</t>
+  </si>
+  <si>
+    <t>Las plataformas aumentan la superficie impermeable en el borde del humedal.</t>
+  </si>
+  <si>
+    <t>Alta: el suelo privado prima sobre la ronda.</t>
+  </si>
+  <si>
+    <t>Coberturas de suelo</t>
+  </si>
+  <si>
+    <t>EDG-46</t>
+  </si>
+  <si>
+    <t>Científica / Monitoreo (Unidireccional)</t>
+  </si>
+  <si>
+    <t>Los observadores registran la presencia de la tingua como indicador de salud del humedal.</t>
+  </si>
+  <si>
+    <t>Baja: aportan datos sin poder de decisión.</t>
+  </si>
+  <si>
+    <t>Listas de avistamientos</t>
+  </si>
+  <si>
+    <t>EDG-47</t>
+  </si>
+  <si>
+    <t>Los conteos de aves terrestres y migratorias sostienen la línea base de biodiversidad.</t>
+  </si>
+  <si>
+    <t>Registros en plataformas de ciencia ciudadana</t>
+  </si>
+  <si>
+    <t>EDG-48</t>
+  </si>
+  <si>
+    <t>Red Comunitaria / Alianza (Bidireccional)</t>
+  </si>
+  <si>
+    <t>La biblioteca presta espacio y difusión a las actividades de la fundación y a la educación ambiental.</t>
+  </si>
+  <si>
+    <t>Baja: relación entre aliados.</t>
+  </si>
+  <si>
+    <t>Agenda cultural y talleres</t>
+  </si>
+  <si>
+    <t>EDG-49</t>
+  </si>
+  <si>
+    <t>Ecológica / Competencia (Unidireccional)</t>
+  </si>
+  <si>
+    <t>El arbolado exótico compite con el saúco por luz y agua en las rondas.</t>
+  </si>
+  <si>
+    <t>Media: crece más rápido que la flora nativa.</t>
+  </si>
+  <si>
+    <t>Inventario de arbolado</t>
+  </si>
+  <si>
+    <t>EDG-50</t>
+  </si>
+  <si>
+    <t>Hábitat / Refugio (Unidireccional)</t>
+  </si>
+  <si>
+    <t>La copa del arbolado exótico sirve de perchas y dormideros a aves generalistas.</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Baja.</t>
+  </si>
+  <si>
+    <t>Observaciones de aves en rondas</t>
+  </si>
+  <si>
+    <t>EDG-51</t>
+  </si>
+  <si>
+    <t>Hidráulica / Conexión (Bidireccional)</t>
+  </si>
+  <si>
+    <t>El canal recibe los excesos del humedal y también le trae aguas lluvias con sedimentos.</t>
+  </si>
+  <si>
+    <t>Alta: la calidad del agua depende de la red externa.</t>
+  </si>
+  <si>
+    <t>Cartografía de drenaje</t>
+  </si>
+  <si>
+    <t>EDG-52</t>
+  </si>
+  <si>
+    <t>Operativa / Mantenimiento (Unidireccional)</t>
+  </si>
+  <si>
+    <t>La EAAB opera y mantiene el canal con dragados periódicos.</t>
+  </si>
+  <si>
+    <t>Alta: decide cuándo y cómo se interviene.</t>
+  </si>
+  <si>
+    <t>Programa de mantenimiento de canales</t>
+  </si>
+  <si>
+    <t>EDG-53</t>
+  </si>
+  <si>
+    <t>Biocultural / Custodia (Unidireccional)</t>
+  </si>
+  <si>
+    <t>El colectivo vigila y restaura el humedal de Techo con jornadas comunitarias.</t>
+  </si>
+  <si>
+    <t>Baja: custodia sin autoridad formal.</t>
+  </si>
+  <si>
+    <t>Jornadas de restauración</t>
+  </si>
+  <si>
+    <t>EDG-54</t>
+  </si>
+  <si>
+    <t>Hábitat / Nidificación (Unidireccional)</t>
+  </si>
+  <si>
+    <t>El humedal de Techo ofrece sitios de nidificación y alimento a la avifauna de la zona.</t>
+  </si>
+  <si>
+    <t>Registros de avifauna</t>
+  </si>
+  <si>
+    <t>EDG-55</t>
+  </si>
+  <si>
+    <t>Urbana / Valorización (Unidireccional)</t>
+  </si>
+  <si>
+    <t>El corredor valoriza el suelo de borde y atrae proyectos de vivienda sobre rondas.</t>
+  </si>
+  <si>
+    <t>Alta: la renta del suelo domina la planeación.</t>
+  </si>
+  <si>
+    <t>Licencias y planes parciales</t>
+  </si>
+  <si>
+    <t>EDG-56</t>
+  </si>
+  <si>
+    <t>Metabólica / Proliferación (Unidireccional)</t>
+  </si>
+  <si>
+    <t>Los lixiviados y aguas de lavado con alta carga orgánica alimentan el crecimiento de bacterias patógenas y cianobacterias en la cubeta hídrica.</t>
+  </si>
+  <si>
+    <t>Extrema: la central genera la carga y las bacterias la expresan en el humedal.</t>
+  </si>
+  <si>
+    <t>Reportes de calidad del agua de la SDA</t>
   </si>
   <si>
     <t>Clave</t>
@@ -2515,7 +2995,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -4251,6 +4731,566 @@
         <v>79</v>
       </c>
       <c r="R31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>393</v>
+      </c>
+      <c r="B32" t="s">
+        <v>394</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E32" t="s">
+        <v>235</v>
+      </c>
+      <c r="F32" t="s">
+        <v>395</v>
+      </c>
+      <c r="G32" t="s">
+        <v>396</v>
+      </c>
+      <c r="H32" t="s">
+        <v>397</v>
+      </c>
+      <c r="I32" t="s">
+        <v>398</v>
+      </c>
+      <c r="J32" t="s">
+        <v>399</v>
+      </c>
+      <c r="K32" t="s">
+        <v>400</v>
+      </c>
+      <c r="L32" t="s">
+        <v>79</v>
+      </c>
+      <c r="M32">
+        <v>4.6395</v>
+      </c>
+      <c r="N32">
+        <v>-74.1625</v>
+      </c>
+      <c r="O32" t="s">
+        <v>79</v>
+      </c>
+      <c r="P32" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>79</v>
+      </c>
+      <c r="R32" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>401</v>
+      </c>
+      <c r="B33" t="s">
+        <v>402</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" t="s">
+        <v>82</v>
+      </c>
+      <c r="E33" t="s">
+        <v>83</v>
+      </c>
+      <c r="F33" t="s">
+        <v>403</v>
+      </c>
+      <c r="G33" t="s">
+        <v>404</v>
+      </c>
+      <c r="H33" t="s">
+        <v>405</v>
+      </c>
+      <c r="I33" t="s">
+        <v>406</v>
+      </c>
+      <c r="J33" t="s">
+        <v>407</v>
+      </c>
+      <c r="K33" t="s">
+        <v>400</v>
+      </c>
+      <c r="L33" t="s">
+        <v>79</v>
+      </c>
+      <c r="M33">
+        <v>4.6315</v>
+      </c>
+      <c r="N33">
+        <v>-74.161</v>
+      </c>
+      <c r="O33" t="s">
+        <v>79</v>
+      </c>
+      <c r="P33" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>79</v>
+      </c>
+      <c r="R33" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>408</v>
+      </c>
+      <c r="B34" t="s">
+        <v>409</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" t="s">
+        <v>105</v>
+      </c>
+      <c r="F34" t="s">
+        <v>410</v>
+      </c>
+      <c r="G34" t="s">
+        <v>411</v>
+      </c>
+      <c r="H34" t="s">
+        <v>412</v>
+      </c>
+      <c r="I34" t="s">
+        <v>413</v>
+      </c>
+      <c r="J34" t="s">
+        <v>414</v>
+      </c>
+      <c r="K34" t="s">
+        <v>400</v>
+      </c>
+      <c r="L34" t="s">
+        <v>79</v>
+      </c>
+      <c r="M34">
+        <v>4.633</v>
+      </c>
+      <c r="N34">
+        <v>-74.1535</v>
+      </c>
+      <c r="O34" t="s">
+        <v>79</v>
+      </c>
+      <c r="P34" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>79</v>
+      </c>
+      <c r="R34" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>415</v>
+      </c>
+      <c r="B35" t="s">
+        <v>416</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>127</v>
+      </c>
+      <c r="E35" t="s">
+        <v>105</v>
+      </c>
+      <c r="F35" t="s">
+        <v>417</v>
+      </c>
+      <c r="G35" t="s">
+        <v>418</v>
+      </c>
+      <c r="H35" t="s">
+        <v>419</v>
+      </c>
+      <c r="I35" t="s">
+        <v>420</v>
+      </c>
+      <c r="J35" t="s">
+        <v>421</v>
+      </c>
+      <c r="K35" t="s">
+        <v>400</v>
+      </c>
+      <c r="L35" t="s">
+        <v>79</v>
+      </c>
+      <c r="M35">
+        <v>4.643</v>
+      </c>
+      <c r="N35">
+        <v>-74.152</v>
+      </c>
+      <c r="O35" t="s">
+        <v>79</v>
+      </c>
+      <c r="P35" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>79</v>
+      </c>
+      <c r="R35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>422</v>
+      </c>
+      <c r="B36" t="s">
+        <v>423</v>
+      </c>
+      <c r="C36" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" t="s">
+        <v>234</v>
+      </c>
+      <c r="E36" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36" t="s">
+        <v>424</v>
+      </c>
+      <c r="G36" t="s">
+        <v>425</v>
+      </c>
+      <c r="H36" t="s">
+        <v>426</v>
+      </c>
+      <c r="I36" t="s">
+        <v>427</v>
+      </c>
+      <c r="J36" t="s">
+        <v>428</v>
+      </c>
+      <c r="K36" t="s">
+        <v>400</v>
+      </c>
+      <c r="L36" t="s">
+        <v>79</v>
+      </c>
+      <c r="M36">
+        <v>4.634</v>
+      </c>
+      <c r="N36">
+        <v>-74.1595</v>
+      </c>
+      <c r="O36" t="s">
+        <v>79</v>
+      </c>
+      <c r="P36" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>79</v>
+      </c>
+      <c r="R36" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>429</v>
+      </c>
+      <c r="B37" t="s">
+        <v>430</v>
+      </c>
+      <c r="C37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" t="s">
+        <v>223</v>
+      </c>
+      <c r="E37" t="s">
+        <v>116</v>
+      </c>
+      <c r="F37" t="s">
+        <v>431</v>
+      </c>
+      <c r="G37" t="s">
+        <v>432</v>
+      </c>
+      <c r="H37" t="s">
+        <v>433</v>
+      </c>
+      <c r="I37" t="s">
+        <v>434</v>
+      </c>
+      <c r="J37" t="s">
+        <v>435</v>
+      </c>
+      <c r="K37" t="s">
+        <v>400</v>
+      </c>
+      <c r="L37" t="s">
+        <v>79</v>
+      </c>
+      <c r="M37">
+        <v>4.6325</v>
+      </c>
+      <c r="N37">
+        <v>-74.1565</v>
+      </c>
+      <c r="O37" t="s">
+        <v>79</v>
+      </c>
+      <c r="P37" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>79</v>
+      </c>
+      <c r="R37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>436</v>
+      </c>
+      <c r="B38" t="s">
+        <v>437</v>
+      </c>
+      <c r="C38" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" t="s">
+        <v>246</v>
+      </c>
+      <c r="E38" t="s">
+        <v>247</v>
+      </c>
+      <c r="F38" t="s">
+        <v>438</v>
+      </c>
+      <c r="G38" t="s">
+        <v>439</v>
+      </c>
+      <c r="H38" t="s">
+        <v>440</v>
+      </c>
+      <c r="I38" t="s">
+        <v>441</v>
+      </c>
+      <c r="J38" t="s">
+        <v>442</v>
+      </c>
+      <c r="K38" t="s">
+        <v>400</v>
+      </c>
+      <c r="L38" t="s">
+        <v>79</v>
+      </c>
+      <c r="M38">
+        <v>4.638</v>
+      </c>
+      <c r="N38">
+        <v>-74.1525</v>
+      </c>
+      <c r="O38" t="s">
+        <v>79</v>
+      </c>
+      <c r="P38" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>79</v>
+      </c>
+      <c r="R38" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>443</v>
+      </c>
+      <c r="B39" t="s">
+        <v>444</v>
+      </c>
+      <c r="C39" t="s">
+        <v>31</v>
+      </c>
+      <c r="D39" t="s">
+        <v>337</v>
+      </c>
+      <c r="E39" t="s">
+        <v>445</v>
+      </c>
+      <c r="F39" t="s">
+        <v>446</v>
+      </c>
+      <c r="G39" t="s">
+        <v>447</v>
+      </c>
+      <c r="H39" t="s">
+        <v>448</v>
+      </c>
+      <c r="I39" t="s">
+        <v>449</v>
+      </c>
+      <c r="J39" t="s">
+        <v>450</v>
+      </c>
+      <c r="K39" t="s">
+        <v>400</v>
+      </c>
+      <c r="L39" t="s">
+        <v>79</v>
+      </c>
+      <c r="M39">
+        <v>4.6405</v>
+      </c>
+      <c r="N39">
+        <v>-74.1495</v>
+      </c>
+      <c r="O39" t="s">
+        <v>79</v>
+      </c>
+      <c r="P39" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>79</v>
+      </c>
+      <c r="R39" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>451</v>
+      </c>
+      <c r="B40" t="s">
+        <v>452</v>
+      </c>
+      <c r="C40" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" t="s">
+        <v>337</v>
+      </c>
+      <c r="E40" t="s">
+        <v>247</v>
+      </c>
+      <c r="F40" t="s">
+        <v>453</v>
+      </c>
+      <c r="G40" t="s">
+        <v>454</v>
+      </c>
+      <c r="H40" t="s">
+        <v>455</v>
+      </c>
+      <c r="I40" t="s">
+        <v>456</v>
+      </c>
+      <c r="J40" t="s">
+        <v>457</v>
+      </c>
+      <c r="K40" t="s">
+        <v>400</v>
+      </c>
+      <c r="L40" t="s">
+        <v>79</v>
+      </c>
+      <c r="M40">
+        <v>4.6535</v>
+      </c>
+      <c r="N40">
+        <v>-74.147</v>
+      </c>
+      <c r="O40" t="s">
+        <v>79</v>
+      </c>
+      <c r="P40" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>79</v>
+      </c>
+      <c r="R40" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>458</v>
+      </c>
+      <c r="B41" t="s">
+        <v>459</v>
+      </c>
+      <c r="C41" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" t="s">
+        <v>337</v>
+      </c>
+      <c r="E41" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" t="s">
+        <v>460</v>
+      </c>
+      <c r="G41" t="s">
+        <v>461</v>
+      </c>
+      <c r="H41" t="s">
+        <v>462</v>
+      </c>
+      <c r="I41" t="s">
+        <v>463</v>
+      </c>
+      <c r="J41" t="s">
+        <v>464</v>
+      </c>
+      <c r="K41" t="s">
+        <v>400</v>
+      </c>
+      <c r="L41" t="s">
+        <v>79</v>
+      </c>
+      <c r="M41">
+        <v>4.645</v>
+      </c>
+      <c r="N41">
+        <v>-74.166</v>
+      </c>
+      <c r="O41" t="s">
+        <v>79</v>
+      </c>
+      <c r="P41" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>79</v>
+      </c>
+      <c r="R41" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4262,7 +5302,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -4270,42 +5310,42 @@
         <v>64</v>
       </c>
       <c r="B1" t="s">
-        <v>393</v>
+        <v>465</v>
       </c>
       <c r="C1" t="s">
-        <v>394</v>
+        <v>466</v>
       </c>
       <c r="D1" t="s">
         <v>36</v>
       </c>
       <c r="E1" t="s">
-        <v>395</v>
+        <v>467</v>
       </c>
       <c r="F1" t="s">
-        <v>396</v>
+        <v>468</v>
       </c>
       <c r="G1" t="s">
-        <v>397</v>
+        <v>469</v>
       </c>
       <c r="H1" t="s">
-        <v>398</v>
+        <v>470</v>
       </c>
       <c r="I1" t="s">
-        <v>399</v>
+        <v>471</v>
       </c>
       <c r="J1" t="s">
-        <v>400</v>
+        <v>472</v>
       </c>
       <c r="K1" t="s">
         <v>72</v>
       </c>
       <c r="L1" t="s">
-        <v>401</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>402</v>
+        <v>474</v>
       </c>
       <c r="B2" t="s">
         <v>125</v>
@@ -4317,13 +5357,13 @@
         <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>403</v>
+        <v>475</v>
       </c>
       <c r="F2" t="s">
-        <v>404</v>
+        <v>476</v>
       </c>
       <c r="G2" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H2">
         <v>3</v>
@@ -4332,18 +5372,18 @@
         <v>79</v>
       </c>
       <c r="J2" t="s">
-        <v>406</v>
+        <v>478</v>
       </c>
       <c r="K2" t="s">
         <v>79</v>
       </c>
       <c r="L2" t="s">
-        <v>407</v>
+        <v>479</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>408</v>
+        <v>480</v>
       </c>
       <c r="B3" t="s">
         <v>125</v>
@@ -4355,13 +5395,13 @@
         <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>409</v>
+        <v>481</v>
       </c>
       <c r="F3" t="s">
-        <v>410</v>
+        <v>482</v>
       </c>
       <c r="G3" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H3">
         <v>3</v>
@@ -4370,18 +5410,18 @@
         <v>79</v>
       </c>
       <c r="J3" t="s">
-        <v>412</v>
+        <v>484</v>
       </c>
       <c r="K3" t="s">
         <v>79</v>
       </c>
       <c r="L3" t="s">
-        <v>413</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>414</v>
+        <v>486</v>
       </c>
       <c r="B4" t="s">
         <v>125</v>
@@ -4393,13 +5433,13 @@
         <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>415</v>
+        <v>487</v>
       </c>
       <c r="F4" t="s">
-        <v>416</v>
+        <v>488</v>
       </c>
       <c r="G4" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -4408,18 +5448,18 @@
         <v>79</v>
       </c>
       <c r="J4" t="s">
-        <v>417</v>
+        <v>489</v>
       </c>
       <c r="K4" t="s">
         <v>79</v>
       </c>
       <c r="L4" t="s">
-        <v>418</v>
+        <v>490</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>419</v>
+        <v>491</v>
       </c>
       <c r="B5" t="s">
         <v>125</v>
@@ -4431,13 +5471,13 @@
         <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>420</v>
+        <v>492</v>
       </c>
       <c r="F5" t="s">
-        <v>421</v>
+        <v>493</v>
       </c>
       <c r="G5" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H5">
         <v>3</v>
@@ -4446,18 +5486,18 @@
         <v>79</v>
       </c>
       <c r="J5" t="s">
-        <v>422</v>
+        <v>494</v>
       </c>
       <c r="K5" t="s">
         <v>79</v>
       </c>
       <c r="L5" t="s">
-        <v>423</v>
+        <v>495</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>424</v>
+        <v>496</v>
       </c>
       <c r="B6" t="s">
         <v>147</v>
@@ -4469,13 +5509,13 @@
         <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>425</v>
+        <v>497</v>
       </c>
       <c r="F6" t="s">
-        <v>426</v>
+        <v>498</v>
       </c>
       <c r="G6" t="s">
-        <v>427</v>
+        <v>499</v>
       </c>
       <c r="H6">
         <v>2</v>
@@ -4484,18 +5524,18 @@
         <v>79</v>
       </c>
       <c r="J6" t="s">
-        <v>428</v>
+        <v>500</v>
       </c>
       <c r="K6" t="s">
         <v>79</v>
       </c>
       <c r="L6" t="s">
-        <v>429</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>430</v>
+        <v>502</v>
       </c>
       <c r="B7" t="s">
         <v>335</v>
@@ -4507,13 +5547,13 @@
         <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>431</v>
+        <v>503</v>
       </c>
       <c r="F7" t="s">
-        <v>432</v>
+        <v>504</v>
       </c>
       <c r="G7" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H7">
         <v>3</v>
@@ -4522,18 +5562,18 @@
         <v>79</v>
       </c>
       <c r="J7" t="s">
-        <v>433</v>
+        <v>505</v>
       </c>
       <c r="K7" t="s">
         <v>79</v>
       </c>
       <c r="L7" t="s">
-        <v>434</v>
+        <v>506</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>435</v>
+        <v>507</v>
       </c>
       <c r="B8" t="s">
         <v>335</v>
@@ -4545,13 +5585,13 @@
         <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>436</v>
+        <v>508</v>
       </c>
       <c r="F8" t="s">
-        <v>437</v>
+        <v>509</v>
       </c>
       <c r="G8" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H8">
         <v>3</v>
@@ -4560,18 +5600,18 @@
         <v>79</v>
       </c>
       <c r="J8" t="s">
-        <v>438</v>
+        <v>510</v>
       </c>
       <c r="K8" t="s">
         <v>79</v>
       </c>
       <c r="L8" t="s">
-        <v>439</v>
+        <v>511</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>440</v>
+        <v>512</v>
       </c>
       <c r="B9" t="s">
         <v>335</v>
@@ -4583,13 +5623,13 @@
         <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>441</v>
+        <v>513</v>
       </c>
       <c r="F9" t="s">
-        <v>442</v>
+        <v>514</v>
       </c>
       <c r="G9" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H9">
         <v>3</v>
@@ -4598,18 +5638,18 @@
         <v>79</v>
       </c>
       <c r="J9" t="s">
-        <v>443</v>
+        <v>515</v>
       </c>
       <c r="K9" t="s">
         <v>79</v>
       </c>
       <c r="L9" t="s">
-        <v>444</v>
+        <v>516</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>445</v>
+        <v>517</v>
       </c>
       <c r="B10" t="s">
         <v>137</v>
@@ -4621,13 +5661,13 @@
         <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>446</v>
+        <v>518</v>
       </c>
       <c r="F10" t="s">
-        <v>447</v>
+        <v>519</v>
       </c>
       <c r="G10" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H10">
         <v>3</v>
@@ -4636,18 +5676,18 @@
         <v>79</v>
       </c>
       <c r="J10" t="s">
-        <v>448</v>
+        <v>520</v>
       </c>
       <c r="K10" t="s">
         <v>79</v>
       </c>
       <c r="L10" t="s">
-        <v>449</v>
+        <v>521</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>450</v>
+        <v>522</v>
       </c>
       <c r="B11" t="s">
         <v>137</v>
@@ -4659,13 +5699,13 @@
         <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>451</v>
+        <v>523</v>
       </c>
       <c r="F11" t="s">
-        <v>452</v>
+        <v>524</v>
       </c>
       <c r="G11" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H11">
         <v>3</v>
@@ -4674,18 +5714,18 @@
         <v>79</v>
       </c>
       <c r="J11" t="s">
-        <v>453</v>
+        <v>525</v>
       </c>
       <c r="K11" t="s">
         <v>79</v>
       </c>
       <c r="L11" t="s">
-        <v>454</v>
+        <v>526</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>455</v>
+        <v>527</v>
       </c>
       <c r="B12" t="s">
         <v>80</v>
@@ -4697,13 +5737,13 @@
         <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>456</v>
+        <v>528</v>
       </c>
       <c r="F12" t="s">
-        <v>457</v>
+        <v>529</v>
       </c>
       <c r="G12" t="s">
-        <v>427</v>
+        <v>499</v>
       </c>
       <c r="H12">
         <v>2</v>
@@ -4712,18 +5752,18 @@
         <v>79</v>
       </c>
       <c r="J12" t="s">
-        <v>458</v>
+        <v>530</v>
       </c>
       <c r="K12" t="s">
         <v>79</v>
       </c>
       <c r="L12" t="s">
-        <v>459</v>
+        <v>531</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>460</v>
+        <v>532</v>
       </c>
       <c r="B13" t="s">
         <v>80</v>
@@ -4735,13 +5775,13 @@
         <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>461</v>
+        <v>533</v>
       </c>
       <c r="F13" t="s">
-        <v>462</v>
+        <v>534</v>
       </c>
       <c r="G13" t="s">
-        <v>427</v>
+        <v>499</v>
       </c>
       <c r="H13">
         <v>2</v>
@@ -4750,18 +5790,18 @@
         <v>79</v>
       </c>
       <c r="J13" t="s">
-        <v>463</v>
+        <v>535</v>
       </c>
       <c r="K13" t="s">
         <v>79</v>
       </c>
       <c r="L13" t="s">
-        <v>464</v>
+        <v>536</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>465</v>
+        <v>537</v>
       </c>
       <c r="B14" t="s">
         <v>92</v>
@@ -4773,13 +5813,13 @@
         <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>466</v>
+        <v>538</v>
       </c>
       <c r="F14" t="s">
-        <v>467</v>
+        <v>539</v>
       </c>
       <c r="G14" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H14">
         <v>3</v>
@@ -4788,18 +5828,18 @@
         <v>79</v>
       </c>
       <c r="J14" t="s">
-        <v>468</v>
+        <v>540</v>
       </c>
       <c r="K14" t="s">
         <v>79</v>
       </c>
       <c r="L14" t="s">
-        <v>469</v>
+        <v>541</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>470</v>
+        <v>542</v>
       </c>
       <c r="B15" t="s">
         <v>92</v>
@@ -4811,13 +5851,13 @@
         <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>471</v>
+        <v>543</v>
       </c>
       <c r="F15" t="s">
-        <v>472</v>
+        <v>544</v>
       </c>
       <c r="G15" t="s">
-        <v>473</v>
+        <v>545</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -4826,18 +5866,18 @@
         <v>79</v>
       </c>
       <c r="J15" t="s">
-        <v>474</v>
+        <v>546</v>
       </c>
       <c r="K15" t="s">
         <v>79</v>
       </c>
       <c r="L15" t="s">
-        <v>475</v>
+        <v>547</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>476</v>
+        <v>548</v>
       </c>
       <c r="B16" t="s">
         <v>103</v>
@@ -4849,13 +5889,13 @@
         <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>477</v>
+        <v>549</v>
       </c>
       <c r="F16" t="s">
-        <v>478</v>
+        <v>550</v>
       </c>
       <c r="G16" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H16">
         <v>3</v>
@@ -4864,18 +5904,18 @@
         <v>79</v>
       </c>
       <c r="J16" t="s">
-        <v>479</v>
+        <v>551</v>
       </c>
       <c r="K16" t="s">
         <v>79</v>
       </c>
       <c r="L16" t="s">
-        <v>480</v>
+        <v>552</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>481</v>
+        <v>553</v>
       </c>
       <c r="B17" t="s">
         <v>103</v>
@@ -4887,13 +5927,13 @@
         <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>482</v>
+        <v>554</v>
       </c>
       <c r="F17" t="s">
-        <v>483</v>
+        <v>555</v>
       </c>
       <c r="G17" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H17">
         <v>3</v>
@@ -4902,18 +5942,18 @@
         <v>79</v>
       </c>
       <c r="J17" t="s">
-        <v>484</v>
+        <v>556</v>
       </c>
       <c r="K17" t="s">
         <v>79</v>
       </c>
       <c r="L17" t="s">
-        <v>485</v>
+        <v>557</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>486</v>
+        <v>558</v>
       </c>
       <c r="B18" t="s">
         <v>365</v>
@@ -4925,13 +5965,13 @@
         <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>487</v>
+        <v>559</v>
       </c>
       <c r="F18" t="s">
-        <v>488</v>
+        <v>560</v>
       </c>
       <c r="G18" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H18">
         <v>3</v>
@@ -4940,18 +5980,18 @@
         <v>79</v>
       </c>
       <c r="J18" t="s">
-        <v>489</v>
+        <v>561</v>
       </c>
       <c r="K18" t="s">
         <v>79</v>
       </c>
       <c r="L18" t="s">
-        <v>490</v>
+        <v>562</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>491</v>
+        <v>563</v>
       </c>
       <c r="B19" t="s">
         <v>114</v>
@@ -4963,13 +6003,13 @@
         <v>52</v>
       </c>
       <c r="E19" t="s">
-        <v>492</v>
+        <v>564</v>
       </c>
       <c r="F19" t="s">
-        <v>493</v>
+        <v>565</v>
       </c>
       <c r="G19" t="s">
-        <v>494</v>
+        <v>566</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -4978,18 +6018,18 @@
         <v>79</v>
       </c>
       <c r="J19" t="s">
-        <v>495</v>
+        <v>567</v>
       </c>
       <c r="K19" t="s">
         <v>79</v>
       </c>
       <c r="L19" t="s">
-        <v>496</v>
+        <v>568</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>497</v>
+        <v>569</v>
       </c>
       <c r="B20" t="s">
         <v>167</v>
@@ -5001,13 +6041,13 @@
         <v>56</v>
       </c>
       <c r="E20" t="s">
-        <v>498</v>
+        <v>570</v>
       </c>
       <c r="F20" t="s">
-        <v>499</v>
+        <v>571</v>
       </c>
       <c r="G20" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -5016,18 +6056,18 @@
         <v>79</v>
       </c>
       <c r="J20" t="s">
-        <v>501</v>
+        <v>573</v>
       </c>
       <c r="K20" t="s">
         <v>79</v>
       </c>
       <c r="L20" t="s">
-        <v>502</v>
+        <v>574</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>503</v>
+        <v>575</v>
       </c>
       <c r="B21" t="s">
         <v>167</v>
@@ -5039,13 +6079,13 @@
         <v>52</v>
       </c>
       <c r="E21" t="s">
-        <v>504</v>
+        <v>576</v>
       </c>
       <c r="F21" t="s">
-        <v>505</v>
+        <v>577</v>
       </c>
       <c r="G21" t="s">
-        <v>506</v>
+        <v>578</v>
       </c>
       <c r="H21">
         <v>1</v>
@@ -5054,18 +6094,18 @@
         <v>79</v>
       </c>
       <c r="J21" t="s">
-        <v>507</v>
+        <v>579</v>
       </c>
       <c r="K21" t="s">
         <v>79</v>
       </c>
       <c r="L21" t="s">
-        <v>508</v>
+        <v>580</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>509</v>
+        <v>581</v>
       </c>
       <c r="B22" t="s">
         <v>179</v>
@@ -5077,13 +6117,13 @@
         <v>56</v>
       </c>
       <c r="E22" t="s">
-        <v>510</v>
+        <v>582</v>
       </c>
       <c r="F22" t="s">
-        <v>511</v>
+        <v>583</v>
       </c>
       <c r="G22" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -5092,18 +6132,18 @@
         <v>79</v>
       </c>
       <c r="J22" t="s">
-        <v>512</v>
+        <v>584</v>
       </c>
       <c r="K22" t="s">
         <v>79</v>
       </c>
       <c r="L22" t="s">
-        <v>513</v>
+        <v>585</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>514</v>
+        <v>586</v>
       </c>
       <c r="B23" t="s">
         <v>189</v>
@@ -5115,13 +6155,13 @@
         <v>43</v>
       </c>
       <c r="E23" t="s">
-        <v>515</v>
+        <v>587</v>
       </c>
       <c r="F23" t="s">
-        <v>516</v>
+        <v>588</v>
       </c>
       <c r="G23" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H23">
         <v>3</v>
@@ -5130,18 +6170,18 @@
         <v>79</v>
       </c>
       <c r="J23" t="s">
-        <v>517</v>
+        <v>589</v>
       </c>
       <c r="K23" t="s">
         <v>79</v>
       </c>
       <c r="L23" t="s">
-        <v>518</v>
+        <v>590</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>519</v>
+        <v>591</v>
       </c>
       <c r="B24" t="s">
         <v>200</v>
@@ -5153,13 +6193,13 @@
         <v>48</v>
       </c>
       <c r="E24" t="s">
-        <v>520</v>
+        <v>592</v>
       </c>
       <c r="F24" t="s">
-        <v>521</v>
+        <v>593</v>
       </c>
       <c r="G24" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H24">
         <v>3</v>
@@ -5168,18 +6208,18 @@
         <v>79</v>
       </c>
       <c r="J24" t="s">
-        <v>522</v>
+        <v>594</v>
       </c>
       <c r="K24" t="s">
         <v>79</v>
       </c>
       <c r="L24" t="s">
-        <v>523</v>
+        <v>595</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>524</v>
+        <v>596</v>
       </c>
       <c r="B25" t="s">
         <v>210</v>
@@ -5191,13 +6231,13 @@
         <v>43</v>
       </c>
       <c r="E25" t="s">
-        <v>525</v>
+        <v>597</v>
       </c>
       <c r="F25" t="s">
-        <v>526</v>
+        <v>598</v>
       </c>
       <c r="G25" t="s">
-        <v>494</v>
+        <v>566</v>
       </c>
       <c r="H25">
         <v>1</v>
@@ -5206,18 +6246,18 @@
         <v>79</v>
       </c>
       <c r="J25" t="s">
-        <v>527</v>
+        <v>599</v>
       </c>
       <c r="K25" t="s">
         <v>79</v>
       </c>
       <c r="L25" t="s">
-        <v>528</v>
+        <v>600</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>529</v>
+        <v>601</v>
       </c>
       <c r="B26" t="s">
         <v>221</v>
@@ -5229,13 +6269,13 @@
         <v>56</v>
       </c>
       <c r="E26" t="s">
-        <v>530</v>
+        <v>602</v>
       </c>
       <c r="F26" t="s">
-        <v>531</v>
+        <v>603</v>
       </c>
       <c r="G26" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -5244,18 +6284,18 @@
         <v>79</v>
       </c>
       <c r="J26" t="s">
-        <v>532</v>
+        <v>604</v>
       </c>
       <c r="K26" t="s">
         <v>79</v>
       </c>
       <c r="L26" t="s">
-        <v>533</v>
+        <v>605</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>534</v>
+        <v>606</v>
       </c>
       <c r="B27" t="s">
         <v>232</v>
@@ -5267,13 +6307,13 @@
         <v>56</v>
       </c>
       <c r="E27" t="s">
-        <v>535</v>
+        <v>607</v>
       </c>
       <c r="F27" t="s">
-        <v>536</v>
+        <v>608</v>
       </c>
       <c r="G27" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H27">
         <v>1</v>
@@ -5282,18 +6322,18 @@
         <v>79</v>
       </c>
       <c r="J27" t="s">
-        <v>537</v>
+        <v>609</v>
       </c>
       <c r="K27" t="s">
         <v>79</v>
       </c>
       <c r="L27" t="s">
-        <v>538</v>
+        <v>610</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>539</v>
+        <v>611</v>
       </c>
       <c r="B28" t="s">
         <v>244</v>
@@ -5305,13 +6345,13 @@
         <v>60</v>
       </c>
       <c r="E28" t="s">
-        <v>540</v>
+        <v>612</v>
       </c>
       <c r="F28" t="s">
-        <v>541</v>
+        <v>613</v>
       </c>
       <c r="G28" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H28">
         <v>1</v>
@@ -5320,18 +6360,18 @@
         <v>79</v>
       </c>
       <c r="J28" t="s">
-        <v>542</v>
+        <v>614</v>
       </c>
       <c r="K28" t="s">
         <v>79</v>
       </c>
       <c r="L28" t="s">
-        <v>543</v>
+        <v>615</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>544</v>
+        <v>616</v>
       </c>
       <c r="B29" t="s">
         <v>256</v>
@@ -5343,13 +6383,13 @@
         <v>60</v>
       </c>
       <c r="E29" t="s">
-        <v>545</v>
+        <v>617</v>
       </c>
       <c r="F29" t="s">
-        <v>546</v>
+        <v>618</v>
       </c>
       <c r="G29" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H29">
         <v>1</v>
@@ -5358,18 +6398,18 @@
         <v>79</v>
       </c>
       <c r="J29" t="s">
-        <v>547</v>
+        <v>619</v>
       </c>
       <c r="K29" t="s">
         <v>79</v>
       </c>
       <c r="L29" t="s">
-        <v>548</v>
+        <v>620</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>549</v>
+        <v>621</v>
       </c>
       <c r="B30" t="s">
         <v>295</v>
@@ -5381,13 +6421,13 @@
         <v>60</v>
       </c>
       <c r="E30" t="s">
-        <v>550</v>
+        <v>622</v>
       </c>
       <c r="F30" t="s">
-        <v>551</v>
+        <v>623</v>
       </c>
       <c r="G30" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -5396,18 +6436,18 @@
         <v>79</v>
       </c>
       <c r="J30" t="s">
-        <v>552</v>
+        <v>624</v>
       </c>
       <c r="K30" t="s">
         <v>79</v>
       </c>
       <c r="L30" t="s">
-        <v>553</v>
+        <v>625</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>554</v>
+        <v>626</v>
       </c>
       <c r="B31" t="s">
         <v>265</v>
@@ -5419,13 +6459,13 @@
         <v>60</v>
       </c>
       <c r="E31" t="s">
-        <v>555</v>
+        <v>627</v>
       </c>
       <c r="F31" t="s">
-        <v>556</v>
+        <v>628</v>
       </c>
       <c r="G31" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H31">
         <v>1</v>
@@ -5434,18 +6474,18 @@
         <v>79</v>
       </c>
       <c r="J31" t="s">
-        <v>557</v>
+        <v>629</v>
       </c>
       <c r="K31" t="s">
         <v>79</v>
       </c>
       <c r="L31" t="s">
-        <v>558</v>
+        <v>630</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>559</v>
+        <v>631</v>
       </c>
       <c r="B32" t="s">
         <v>265</v>
@@ -5457,13 +6497,13 @@
         <v>60</v>
       </c>
       <c r="E32" t="s">
-        <v>560</v>
+        <v>632</v>
       </c>
       <c r="F32" t="s">
-        <v>561</v>
+        <v>633</v>
       </c>
       <c r="G32" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -5472,18 +6512,18 @@
         <v>79</v>
       </c>
       <c r="J32" t="s">
-        <v>562</v>
+        <v>634</v>
       </c>
       <c r="K32" t="s">
         <v>79</v>
       </c>
       <c r="L32" t="s">
-        <v>563</v>
+        <v>635</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>564</v>
+        <v>636</v>
       </c>
       <c r="B33" t="s">
         <v>305</v>
@@ -5495,13 +6535,13 @@
         <v>60</v>
       </c>
       <c r="E33" t="s">
-        <v>565</v>
+        <v>637</v>
       </c>
       <c r="F33" t="s">
-        <v>566</v>
+        <v>638</v>
       </c>
       <c r="G33" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H33">
         <v>1</v>
@@ -5510,18 +6550,18 @@
         <v>79</v>
       </c>
       <c r="J33" t="s">
-        <v>567</v>
+        <v>639</v>
       </c>
       <c r="K33" t="s">
         <v>79</v>
       </c>
       <c r="L33" t="s">
-        <v>568</v>
+        <v>640</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>569</v>
+        <v>641</v>
       </c>
       <c r="B34" t="s">
         <v>315</v>
@@ -5533,13 +6573,13 @@
         <v>60</v>
       </c>
       <c r="E34" t="s">
-        <v>570</v>
+        <v>642</v>
       </c>
       <c r="F34" t="s">
-        <v>571</v>
+        <v>643</v>
       </c>
       <c r="G34" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H34">
         <v>1</v>
@@ -5548,18 +6588,18 @@
         <v>79</v>
       </c>
       <c r="J34" t="s">
-        <v>572</v>
+        <v>644</v>
       </c>
       <c r="K34" t="s">
         <v>79</v>
       </c>
       <c r="L34" t="s">
-        <v>573</v>
+        <v>645</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>574</v>
+        <v>646</v>
       </c>
       <c r="B35" t="s">
         <v>315</v>
@@ -5571,13 +6611,13 @@
         <v>39</v>
       </c>
       <c r="E35" t="s">
-        <v>575</v>
+        <v>647</v>
       </c>
       <c r="F35" t="s">
-        <v>576</v>
+        <v>648</v>
       </c>
       <c r="G35" t="s">
-        <v>500</v>
+        <v>572</v>
       </c>
       <c r="H35">
         <v>1</v>
@@ -5586,18 +6626,18 @@
         <v>79</v>
       </c>
       <c r="J35" t="s">
-        <v>577</v>
+        <v>649</v>
       </c>
       <c r="K35" t="s">
         <v>79</v>
       </c>
       <c r="L35" t="s">
-        <v>578</v>
+        <v>650</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>579</v>
+        <v>651</v>
       </c>
       <c r="B36" t="s">
         <v>356</v>
@@ -5609,13 +6649,13 @@
         <v>39</v>
       </c>
       <c r="E36" t="s">
-        <v>580</v>
+        <v>652</v>
       </c>
       <c r="F36" t="s">
-        <v>581</v>
+        <v>653</v>
       </c>
       <c r="G36" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H36">
         <v>3</v>
@@ -5624,18 +6664,18 @@
         <v>79</v>
       </c>
       <c r="J36" t="s">
-        <v>582</v>
+        <v>654</v>
       </c>
       <c r="K36" t="s">
         <v>79</v>
       </c>
       <c r="L36" t="s">
-        <v>583</v>
+        <v>655</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>584</v>
+        <v>656</v>
       </c>
       <c r="B37" t="s">
         <v>346</v>
@@ -5647,13 +6687,13 @@
         <v>48</v>
       </c>
       <c r="E37" t="s">
-        <v>585</v>
+        <v>657</v>
       </c>
       <c r="F37" t="s">
-        <v>586</v>
+        <v>658</v>
       </c>
       <c r="G37" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="H37">
         <v>3</v>
@@ -5662,18 +6702,18 @@
         <v>79</v>
       </c>
       <c r="J37" t="s">
-        <v>587</v>
+        <v>659</v>
       </c>
       <c r="K37" t="s">
         <v>79</v>
       </c>
       <c r="L37" t="s">
-        <v>588</v>
+        <v>660</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>589</v>
+        <v>661</v>
       </c>
       <c r="B38" t="s">
         <v>346</v>
@@ -5685,13 +6725,13 @@
         <v>48</v>
       </c>
       <c r="E38" t="s">
-        <v>590</v>
+        <v>662</v>
       </c>
       <c r="F38" t="s">
-        <v>591</v>
+        <v>663</v>
       </c>
       <c r="G38" t="s">
-        <v>411</v>
+        <v>483</v>
       </c>
       <c r="H38">
         <v>3</v>
@@ -5700,18 +6740,18 @@
         <v>79</v>
       </c>
       <c r="J38" t="s">
-        <v>592</v>
+        <v>664</v>
       </c>
       <c r="K38" t="s">
         <v>79</v>
       </c>
       <c r="L38" t="s">
-        <v>593</v>
+        <v>665</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>594</v>
+        <v>666</v>
       </c>
       <c r="B39" t="s">
         <v>157</v>
@@ -5723,13 +6763,13 @@
         <v>48</v>
       </c>
       <c r="E39" t="s">
-        <v>595</v>
+        <v>667</v>
       </c>
       <c r="F39" t="s">
-        <v>596</v>
+        <v>668</v>
       </c>
       <c r="G39" t="s">
-        <v>427</v>
+        <v>499</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -5738,13 +6778,697 @@
         <v>79</v>
       </c>
       <c r="J39" t="s">
-        <v>597</v>
+        <v>669</v>
       </c>
       <c r="K39" t="s">
         <v>79</v>
       </c>
       <c r="L39" t="s">
-        <v>598</v>
+        <v>670</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>671</v>
+      </c>
+      <c r="B40" t="s">
+        <v>393</v>
+      </c>
+      <c r="C40" t="s">
+        <v>365</v>
+      </c>
+      <c r="D40" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" t="s">
+        <v>672</v>
+      </c>
+      <c r="F40" t="s">
+        <v>673</v>
+      </c>
+      <c r="G40" t="s">
+        <v>499</v>
+      </c>
+      <c r="H40">
+        <v>2</v>
+      </c>
+      <c r="I40" t="s">
+        <v>79</v>
+      </c>
+      <c r="J40" t="s">
+        <v>674</v>
+      </c>
+      <c r="K40" t="s">
+        <v>79</v>
+      </c>
+      <c r="L40" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>676</v>
+      </c>
+      <c r="B41" t="s">
+        <v>393</v>
+      </c>
+      <c r="C41" t="s">
+        <v>375</v>
+      </c>
+      <c r="D41" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" t="s">
+        <v>677</v>
+      </c>
+      <c r="F41" t="s">
+        <v>678</v>
+      </c>
+      <c r="G41" t="s">
+        <v>566</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41" t="s">
+        <v>79</v>
+      </c>
+      <c r="J41" t="s">
+        <v>679</v>
+      </c>
+      <c r="K41" t="s">
+        <v>79</v>
+      </c>
+      <c r="L41" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>681</v>
+      </c>
+      <c r="B42" t="s">
+        <v>401</v>
+      </c>
+      <c r="C42" t="s">
+        <v>200</v>
+      </c>
+      <c r="D42" t="s">
+        <v>52</v>
+      </c>
+      <c r="E42" t="s">
+        <v>682</v>
+      </c>
+      <c r="F42" t="s">
+        <v>683</v>
+      </c>
+      <c r="G42" t="s">
+        <v>566</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42" t="s">
+        <v>79</v>
+      </c>
+      <c r="J42" t="s">
+        <v>684</v>
+      </c>
+      <c r="K42" t="s">
+        <v>79</v>
+      </c>
+      <c r="L42" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>686</v>
+      </c>
+      <c r="B43" t="s">
+        <v>401</v>
+      </c>
+      <c r="C43" t="s">
+        <v>125</v>
+      </c>
+      <c r="D43" t="s">
+        <v>52</v>
+      </c>
+      <c r="E43" t="s">
+        <v>687</v>
+      </c>
+      <c r="F43" t="s">
+        <v>688</v>
+      </c>
+      <c r="G43" t="s">
+        <v>499</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
+      </c>
+      <c r="I43" t="s">
+        <v>79</v>
+      </c>
+      <c r="J43" t="s">
+        <v>689</v>
+      </c>
+      <c r="K43" t="s">
+        <v>79</v>
+      </c>
+      <c r="L43" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>691</v>
+      </c>
+      <c r="B44" t="s">
+        <v>408</v>
+      </c>
+      <c r="C44" t="s">
+        <v>335</v>
+      </c>
+      <c r="D44" t="s">
+        <v>52</v>
+      </c>
+      <c r="E44" t="s">
+        <v>692</v>
+      </c>
+      <c r="F44" t="s">
+        <v>693</v>
+      </c>
+      <c r="G44" t="s">
+        <v>499</v>
+      </c>
+      <c r="H44">
+        <v>2</v>
+      </c>
+      <c r="I44" t="s">
+        <v>79</v>
+      </c>
+      <c r="J44" t="s">
+        <v>694</v>
+      </c>
+      <c r="K44" t="s">
+        <v>79</v>
+      </c>
+      <c r="L44" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>696</v>
+      </c>
+      <c r="B45" t="s">
+        <v>415</v>
+      </c>
+      <c r="C45" t="s">
+        <v>335</v>
+      </c>
+      <c r="D45" t="s">
+        <v>43</v>
+      </c>
+      <c r="E45" t="s">
+        <v>697</v>
+      </c>
+      <c r="F45" t="s">
+        <v>698</v>
+      </c>
+      <c r="G45" t="s">
+        <v>499</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45" t="s">
+        <v>79</v>
+      </c>
+      <c r="J45" t="s">
+        <v>699</v>
+      </c>
+      <c r="K45" t="s">
+        <v>79</v>
+      </c>
+      <c r="L45" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>701</v>
+      </c>
+      <c r="B46" t="s">
+        <v>415</v>
+      </c>
+      <c r="C46" t="s">
+        <v>346</v>
+      </c>
+      <c r="D46" t="s">
+        <v>43</v>
+      </c>
+      <c r="E46" t="s">
+        <v>702</v>
+      </c>
+      <c r="F46" t="s">
+        <v>703</v>
+      </c>
+      <c r="G46" t="s">
+        <v>483</v>
+      </c>
+      <c r="H46">
+        <v>3</v>
+      </c>
+      <c r="I46" t="s">
+        <v>79</v>
+      </c>
+      <c r="J46" t="s">
+        <v>704</v>
+      </c>
+      <c r="K46" t="s">
+        <v>79</v>
+      </c>
+      <c r="L46" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>706</v>
+      </c>
+      <c r="B47" t="s">
+        <v>422</v>
+      </c>
+      <c r="C47" t="s">
+        <v>275</v>
+      </c>
+      <c r="D47" t="s">
+        <v>56</v>
+      </c>
+      <c r="E47" t="s">
+        <v>707</v>
+      </c>
+      <c r="F47" t="s">
+        <v>708</v>
+      </c>
+      <c r="G47" t="s">
+        <v>566</v>
+      </c>
+      <c r="H47">
+        <v>1</v>
+      </c>
+      <c r="I47" t="s">
+        <v>79</v>
+      </c>
+      <c r="J47" t="s">
+        <v>709</v>
+      </c>
+      <c r="K47" t="s">
+        <v>79</v>
+      </c>
+      <c r="L47" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>711</v>
+      </c>
+      <c r="B48" t="s">
+        <v>422</v>
+      </c>
+      <c r="C48" t="s">
+        <v>295</v>
+      </c>
+      <c r="D48" t="s">
+        <v>56</v>
+      </c>
+      <c r="E48" t="s">
+        <v>707</v>
+      </c>
+      <c r="F48" t="s">
+        <v>712</v>
+      </c>
+      <c r="G48" t="s">
+        <v>566</v>
+      </c>
+      <c r="H48">
+        <v>1</v>
+      </c>
+      <c r="I48" t="s">
+        <v>79</v>
+      </c>
+      <c r="J48" t="s">
+        <v>709</v>
+      </c>
+      <c r="K48" t="s">
+        <v>79</v>
+      </c>
+      <c r="L48" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>714</v>
+      </c>
+      <c r="B49" t="s">
+        <v>429</v>
+      </c>
+      <c r="C49" t="s">
+        <v>167</v>
+      </c>
+      <c r="D49" t="s">
+        <v>56</v>
+      </c>
+      <c r="E49" t="s">
+        <v>715</v>
+      </c>
+      <c r="F49" t="s">
+        <v>716</v>
+      </c>
+      <c r="G49" t="s">
+        <v>566</v>
+      </c>
+      <c r="H49">
+        <v>1</v>
+      </c>
+      <c r="I49" t="s">
+        <v>79</v>
+      </c>
+      <c r="J49" t="s">
+        <v>717</v>
+      </c>
+      <c r="K49" t="s">
+        <v>79</v>
+      </c>
+      <c r="L49" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>719</v>
+      </c>
+      <c r="B50" t="s">
+        <v>436</v>
+      </c>
+      <c r="C50" t="s">
+        <v>244</v>
+      </c>
+      <c r="D50" t="s">
+        <v>48</v>
+      </c>
+      <c r="E50" t="s">
+        <v>720</v>
+      </c>
+      <c r="F50" t="s">
+        <v>721</v>
+      </c>
+      <c r="G50" t="s">
+        <v>566</v>
+      </c>
+      <c r="H50">
+        <v>1</v>
+      </c>
+      <c r="I50" t="s">
+        <v>79</v>
+      </c>
+      <c r="J50" t="s">
+        <v>722</v>
+      </c>
+      <c r="K50" t="s">
+        <v>79</v>
+      </c>
+      <c r="L50" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>724</v>
+      </c>
+      <c r="B51" t="s">
+        <v>436</v>
+      </c>
+      <c r="C51" t="s">
+        <v>295</v>
+      </c>
+      <c r="D51" t="s">
+        <v>60</v>
+      </c>
+      <c r="E51" t="s">
+        <v>725</v>
+      </c>
+      <c r="F51" t="s">
+        <v>726</v>
+      </c>
+      <c r="G51" t="s">
+        <v>727</v>
+      </c>
+      <c r="H51">
+        <v>1</v>
+      </c>
+      <c r="I51" t="s">
+        <v>79</v>
+      </c>
+      <c r="J51" t="s">
+        <v>728</v>
+      </c>
+      <c r="K51" t="s">
+        <v>79</v>
+      </c>
+      <c r="L51" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>730</v>
+      </c>
+      <c r="B52" t="s">
+        <v>443</v>
+      </c>
+      <c r="C52" t="s">
+        <v>375</v>
+      </c>
+      <c r="D52" t="s">
+        <v>39</v>
+      </c>
+      <c r="E52" t="s">
+        <v>731</v>
+      </c>
+      <c r="F52" t="s">
+        <v>732</v>
+      </c>
+      <c r="G52" t="s">
+        <v>499</v>
+      </c>
+      <c r="H52">
+        <v>2</v>
+      </c>
+      <c r="I52" t="s">
+        <v>79</v>
+      </c>
+      <c r="J52" t="s">
+        <v>733</v>
+      </c>
+      <c r="K52" t="s">
+        <v>79</v>
+      </c>
+      <c r="L52" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>735</v>
+      </c>
+      <c r="B53" t="s">
+        <v>103</v>
+      </c>
+      <c r="C53" t="s">
+        <v>443</v>
+      </c>
+      <c r="D53" t="s">
+        <v>56</v>
+      </c>
+      <c r="E53" t="s">
+        <v>736</v>
+      </c>
+      <c r="F53" t="s">
+        <v>737</v>
+      </c>
+      <c r="G53" t="s">
+        <v>566</v>
+      </c>
+      <c r="H53">
+        <v>1</v>
+      </c>
+      <c r="I53" t="s">
+        <v>79</v>
+      </c>
+      <c r="J53" t="s">
+        <v>738</v>
+      </c>
+      <c r="K53" t="s">
+        <v>79</v>
+      </c>
+      <c r="L53" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>740</v>
+      </c>
+      <c r="B54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C54" t="s">
+        <v>451</v>
+      </c>
+      <c r="D54" t="s">
+        <v>56</v>
+      </c>
+      <c r="E54" t="s">
+        <v>741</v>
+      </c>
+      <c r="F54" t="s">
+        <v>742</v>
+      </c>
+      <c r="G54" t="s">
+        <v>566</v>
+      </c>
+      <c r="H54">
+        <v>1</v>
+      </c>
+      <c r="I54" t="s">
+        <v>79</v>
+      </c>
+      <c r="J54" t="s">
+        <v>743</v>
+      </c>
+      <c r="K54" t="s">
+        <v>79</v>
+      </c>
+      <c r="L54" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>745</v>
+      </c>
+      <c r="B55" t="s">
+        <v>451</v>
+      </c>
+      <c r="C55" t="s">
+        <v>295</v>
+      </c>
+      <c r="D55" t="s">
+        <v>60</v>
+      </c>
+      <c r="E55" t="s">
+        <v>746</v>
+      </c>
+      <c r="F55" t="s">
+        <v>747</v>
+      </c>
+      <c r="G55" t="s">
+        <v>566</v>
+      </c>
+      <c r="H55">
+        <v>1</v>
+      </c>
+      <c r="I55" t="s">
+        <v>79</v>
+      </c>
+      <c r="J55" t="s">
+        <v>728</v>
+      </c>
+      <c r="K55" t="s">
+        <v>79</v>
+      </c>
+      <c r="L55" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>749</v>
+      </c>
+      <c r="B56" t="s">
+        <v>458</v>
+      </c>
+      <c r="C56" t="s">
+        <v>137</v>
+      </c>
+      <c r="D56" t="s">
+        <v>43</v>
+      </c>
+      <c r="E56" t="s">
+        <v>750</v>
+      </c>
+      <c r="F56" t="s">
+        <v>751</v>
+      </c>
+      <c r="G56" t="s">
+        <v>499</v>
+      </c>
+      <c r="H56">
+        <v>2</v>
+      </c>
+      <c r="I56" t="s">
+        <v>79</v>
+      </c>
+      <c r="J56" t="s">
+        <v>752</v>
+      </c>
+      <c r="K56" t="s">
+        <v>79</v>
+      </c>
+      <c r="L56" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>754</v>
+      </c>
+      <c r="B57" t="s">
+        <v>125</v>
+      </c>
+      <c r="C57" t="s">
+        <v>325</v>
+      </c>
+      <c r="D57" t="s">
+        <v>39</v>
+      </c>
+      <c r="E57" t="s">
+        <v>755</v>
+      </c>
+      <c r="F57" t="s">
+        <v>756</v>
+      </c>
+      <c r="G57" t="s">
+        <v>483</v>
+      </c>
+      <c r="H57">
+        <v>3</v>
+      </c>
+      <c r="I57" t="s">
+        <v>79</v>
+      </c>
+      <c r="J57" t="s">
+        <v>757</v>
+      </c>
+      <c r="K57" t="s">
+        <v>79</v>
+      </c>
+      <c r="L57" t="s">
+        <v>758</v>
       </c>
     </row>
   </sheetData>
@@ -5760,90 +7484,90 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>599</v>
+        <v>759</v>
       </c>
       <c r="B1" t="s">
-        <v>600</v>
+        <v>760</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>601</v>
+        <v>761</v>
       </c>
       <c r="B2" t="s">
-        <v>602</v>
+        <v>762</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>603</v>
+        <v>763</v>
       </c>
       <c r="B3" t="s">
-        <v>604</v>
+        <v>764</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>605</v>
+        <v>765</v>
       </c>
       <c r="B4" t="s">
-        <v>606</v>
+        <v>766</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>607</v>
+        <v>767</v>
       </c>
       <c r="B5" t="s">
-        <v>608</v>
+        <v>768</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>609</v>
+        <v>769</v>
       </c>
       <c r="B6" t="s">
-        <v>610</v>
+        <v>770</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>611</v>
+        <v>771</v>
       </c>
       <c r="B7" t="s">
-        <v>612</v>
+        <v>772</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>613</v>
+        <v>773</v>
       </c>
       <c r="B8" t="s">
-        <v>614</v>
+        <v>774</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>615</v>
+        <v>775</v>
       </c>
       <c r="B9" t="s">
-        <v>616</v>
+        <v>776</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>617</v>
+        <v>777</v>
       </c>
       <c r="B10" t="s">
-        <v>618</v>
+        <v>778</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>619</v>
+        <v>779</v>
       </c>
       <c r="B11" t="s">
-        <v>620</v>
+        <v>780</v>
       </c>
     </row>
   </sheetData>

</xml_diff>